<commit_message>
Fix bubble reader and OCR extraction
</commit_message>
<xml_diff>
--- a/output/reports_export.xlsx
+++ b/output/reports_export.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,7 +556,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-29T12:11:36.162920</t>
+          <t>2026-05-30T00:04:44.605719</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>‘EPIY DCE Und lan res</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -581,11 +581,11 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3/16</t>
+          <t>4/16</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>18.8</v>
+        <v>25</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -593,15 +593,19 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
         <v>11</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>A</t>
@@ -609,7 +613,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -619,7 +623,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -629,17 +633,13 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -649,13 +649,17 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -665,19 +669,19 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-29T12:17:44.898491</t>
+          <t>2026-05-30T00:05:36.876312</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -687,50 +691,50 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>18.8</v>
+        <v>62.5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="n">
-        <v>11</v>
-      </c>
       <c r="K3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -750,30 +754,26 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>B</t>
@@ -781,12 +781,12 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -798,7 +798,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-29T12:27:45.586701</t>
+          <t>2026-05-30T00:55:41.144097</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -808,50 +808,50 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>18.8</v>
+        <v>62.5</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J4" t="n">
         <v>3</v>
       </c>
-      <c r="J4" t="n">
-        <v>11</v>
-      </c>
       <c r="K4" t="n">
-        <v>2</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -871,30 +871,26 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr">
         <is>
           <t>B</t>
@@ -902,12 +898,12 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -919,7 +915,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-29T12:57:09.530640</t>
+          <t>2026-05-30T01:31:44.573364</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -929,52 +925,52 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>A</t>
@@ -985,10 +981,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
@@ -997,38 +997,42 @@
           <t>B</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-29T13:01:48.020583</t>
+          <t>2026-05-30T01:56:35.673391</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1038,52 +1042,52 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>A</t>
@@ -1094,10 +1098,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
@@ -1106,38 +1114,42 @@
           <t>B</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-29T13:05:07.072582</t>
+          <t>2026-05-30T02:02:19.235173</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1147,51 +1159,47 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>4/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J7" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>B</t>
@@ -1204,7 +1212,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1214,7 +1222,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
@@ -1223,11 +1231,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
           <t>C</t>
@@ -1235,34 +1239,34 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-29T13:09:26.782118</t>
+          <t>2026-05-30T03:48:34.831462</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1272,51 +1276,47 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>4/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J8" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>B</t>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
@@ -1348,11 +1348,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr">
         <is>
           <t>C</t>
@@ -1360,34 +1356,34 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-29T13:35:51.378071</t>
+          <t>2026-05-30T04:07:03.007258</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1397,51 +1393,47 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>it ohdo</t>
+          <t>s BSE JFA2Y- O4F ae iad</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AI Quiz SP2026 Set-A</t>
+          <t>AI Quiz SP2026 Set-B</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>4/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>25</v>
+        <v>62.5</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J9" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>B</t>
@@ -1454,7 +1446,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1464,7 +1456,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
@@ -1473,11 +1465,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr">
         <is>
           <t>C</t>
@@ -1485,27 +1473,261 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-30T04:07:25.604610</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>s BSE JFA2Y- O4F ae iad</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AI Quiz SP2026 Set-B</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>10</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-30T04:07:55.821115</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>s BSE JFA2Y- O4F ae iad</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AI Quiz SP2026 Set-B</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>

</xml_diff>